<commit_message>
add: update final assessment file for Module 5 on Data Modelling
</commit_message>
<xml_diff>
--- a/03-intermediate-2/material_curso/modulo-05/assessment/C3-W5-Final-Assessment.xlsx
+++ b/03-intermediate-2/material_curso/modulo-05/assessment/C3-W5-Final-Assessment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jorge\Proyectos\ExcelLearning\03-intermediate-2\material_curso\modulo-05\assessment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65372AB2-C57E-45D3-8635-A8C00F50AEBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97E5E988-3859-43DA-A091-4BBFAD601D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="6" r:id="rId1"/>
@@ -2760,7 +2760,7 @@
         <v>19</v>
       </c>
       <c r="B38" s="38">
-        <v>1</v>
+        <v>2.8914174009120024</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="B39" s="61">
         <f>(240 - 30*B38)*1000*B38</f>
-        <v>210000</v>
+        <v>443131.33862997906</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="B40" s="18">
         <f>(120 + 8*B38)*1000</f>
-        <v>128000</v>
+        <v>143131.339207296</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="B41" s="40">
         <f>B39-B40</f>
-        <v>82000</v>
+        <v>299999.99942268303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>